<commit_message>
test(regression): integrations под-блок 2 — notifications + view; закрыт WH-pending
Notifications (/me/notifications) + order view (POST /orders/{id}/view), API-INT-025…048:
27 passed (24 кейса + 3 WH-закрытия). Уведомления — PUSH-инбокс перевозчика после
bid-request; view — трекинг просмотра (TRANSPORT_ADMIN/DRIVER, не идемпотентен).

Закрыт cross-module pending:
- WH-130/131/134 (dispatch-log агрегация/сортировка/фильтрация) — сняты pending, покрыты
  через view-события (несколько view → viewCount; TRANSPORT>DRIVER сортировка; удалённый
  получатель отброшен). Warehouse теперь 138/138 = 100%. pending по набору = 0.

Расхождения → триаж (устаревшие кейсы): INT-036 (невалидный UUID в пути → BAD_REQUEST,
не error.bad-request), INT-031 (поле счётчика — unread, не count). Синхронизировано.

ИТОГО 830/1497 = 55.4%. Осталось в модуле: SMS (3) · 1С (4) · files (5) · blacklist (6).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testcases/manzil-api-testcases.xlsx
+++ b/docs/testcases/manzil-api-testcases.xlsx
@@ -37300,7 +37300,7 @@
       <c r="I131" s="3" t="inlineStr"/>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>api|positive · automation:pending 2026-07-23: нужен хелпер провизининга dispatch/view-событий (агрегация viewCount=max по нескольким строкам получателя) — Фаза 4b integrations</t>
+          <t>api|positive · automation:pending 2026-07-23: нужен хелпер провизининга dispatch/view-событий (агрегация viewCount=max по нескольким строкам получателя) — Фаза 4b integrations · закрыто 2026-07-23: view-события (POST /orders/{id}/view) в test_int_notifications.py</t>
         </is>
       </c>
     </row>
@@ -37349,7 +37349,7 @@
       <c r="I132" s="3" t="inlineStr"/>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>api|positive · automation:pending 2026-07-23: нужен хелпер провизининга dispatch/view-событий (сортировка TRANSPORT&gt;DRIVER, viewCount desc) — Фаза 4b integrations</t>
+          <t>api|positive · automation:pending 2026-07-23: нужен хелпер провизининга dispatch/view-событий (сортировка TRANSPORT&gt;DRIVER, viewCount desc) — Фаза 4b integrations · закрыто 2026-07-23: view-события (POST /orders/{id}/view) в test_int_notifications.py</t>
         </is>
       </c>
     </row>
@@ -37493,7 +37493,7 @@
       <c r="I135" s="3" t="inlineStr"/>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t>api|positive · automation:pending 2026-07-23: нужен хелпер провизининга dispatch/view-событий (фильтрация удалённого получателя) — Фаза 4b integrations</t>
+          <t>api|positive · automation:pending 2026-07-23: нужен хелпер провизининга dispatch/view-событий (фильтрация удалённого получателя) — Фаза 4b integrations · закрыто 2026-07-23: view-события (POST /orders/{id}/view) в test_int_notifications.py</t>
         </is>
       </c>
     </row>
@@ -39242,7 +39242,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; в теле поле count — число непрочитанных PUSH-уведомлений пользователя (значение для бейджа).</t>
+          <t>HTTP 200; в теле поле поле unread — число непрочитанных PUSH-уведомлений пользователя (значение для бейджа).</t>
         </is>
       </c>
       <c r="H32" s="9" t="inlineStr">
@@ -39253,7 +39253,7 @@
       <c r="I32" s="3" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>api|positive</t>
+          <t>api|positive · уточнено 2026-07-23: поле счётчика — unread (не count)</t>
         </is>
       </c>
     </row>
@@ -39483,7 +39483,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>HTTP 400, code=error.bad-request — значение в пути не является корректным UUID.</t>
+          <t>HTTP 400, code=BAD_REQUEST — значение в пути не является корректным UUID.</t>
         </is>
       </c>
       <c r="H37" s="10" t="inlineStr">
@@ -39494,7 +39494,7 @@
       <c r="I37" s="3" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>api|validation</t>
+          <t>api|validation · уточнено 2026-07-23: невалидный UUID в пути → framework BAD_REQUEST</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(regression): integrations под-блок 3 — SMS blast + sms-logs (INT-060…080)
22 теста: рассылка bid-request (204/eligibility/debounce/tenancy) + журнал
(фильтры/date-range/RBAC/tenancy) + capability-матрица SMS_BLAST/SMS_JOURNAL.
Тест-сторож `test_sms_config_sentinel_noop`: подтверждает dev no-op (все строки
result=SKIPPED, ни одной SENT) — упадёт ПЕРВЫМ, если dev когда-нибудь получит
рабочий Aliyun-провайдер. Реальных SMS не шлётся: dev unconfigured + фильтр +86.

Уточнено по факту (JSON синхронизирован): роль без SMS_BLAST/SMS_JOURNAL —
SHIPPER_OPERATOR (у ADMIN/MANAGER/DISPATCHER обе capability по умолчанию,
RoleCapabilityDefaults). Поле строки журнала — result (SKIPPED/SENT), не status.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testcases/manzil-api-testcases.xlsx
+++ b/docs/testcases/manzil-api-testcases.xlsx
@@ -40821,7 +40821,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Выполнен вход под SHIPPER_ADMIN, у которого нет capability SMS_BLAST.</t>
+          <t>Выполнен вход под SHIPPER_OPERATOR (роль без capability SMS_BLAST по умолчанию); заказ в статусе PUBLISHED.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -40842,7 +40842,7 @@
       <c r="I65" s="3" t="inlineStr"/>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>api|capability</t>
+          <t>api|capability · уточнено по факту: SMS_BLAST есть по умолчанию у ADMIN/MANAGER/DISPATCHER — роль без неё это OPERATOR (2026-07-23)</t>
         </is>
       </c>
     </row>
@@ -41398,7 +41398,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Выполнен вход под SHIPPER_ADMIN, у которого нет capability SMS_JOURNAL.</t>
+          <t>Выполнен вход под SHIPPER_OPERATOR (роль без capability SMS_JOURNAL по умолчанию).</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -41419,7 +41419,7 @@
       <c r="I77" s="3" t="inlineStr"/>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>api|capability</t>
+          <t>api|capability · уточнено по факту: SMS_JOURNAL есть по умолчанию у ADMIN/MANAGER/DISPATCHER — роль без неё это OPERATOR (2026-07-23)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(cases): регистрация MNZL-269 — 70 API-кейсов (API-REG) + 7 web-SA + книги 1574
docs/testcases/api/08_registration_reset_public.json — API-REG-001…070: регистрация
ТК/водителя через OTP, сброс пароля, публичная лента грузов, верификация перевозчиков.
WEB-SA-066…072 — вкладки/карточки согласования в «Партнёрах».

Флаги автоматизации (снято пробой публичного dev): класс B (verify→complete→gating→
reset, 29) — automation:pending, тест-OTP-код на публичном dev выключен, verify недостижим;
API-REG-012/013 (реальный SMS) — automation:manual. REG-064 expected уточнён по факту
(from/to={cityName,country}).

Книги пересобраны 1497→1574 (build_full_book.py: секция 08).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testcases/manzil-api-testcases.xlsx
+++ b/docs/testcases/manzil-api-testcases.xlsx
@@ -53074,7 +53074,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>В записи ровно: id (внутренний числовой), cargoType, loadDate, vehicleTypeName, driversCount, from/to (только регион). НЕТ: цен и ставок, названия/идентификаторов отправителя, номера заказа (displayNumber), адресов складов, заметок. Утечка любого из этих полей — баг безопасности.</t>
+          <t>В записи ровно: id (внутренний числовой), cargoType, loadDate, vehicleTypeName, driversCount, from/to — каждый как {cityName, country} (город и страна, без точного адреса/склада). НЕТ: цен и ставок, названия/идентификаторов отправителя, номера заказа (displayNumber), адресов складов, заметок. Утечка любого из этих полей — баг безопасности.</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
@@ -53085,7 +53085,7 @@
       <c r="I65" s="3" t="inlineStr"/>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>api|positive|security</t>
+          <t>api|positive|security · уточнено по фактическому контракту 2026-07-24 (from/to={cityName,country})</t>
         </is>
       </c>
     </row>

</xml_diff>